<commit_message>
Fixed: - Updated version parameter to tests
</commit_message>
<xml_diff>
--- a/tests/reference_data/example_scenario.xlsx
+++ b/tests/reference_data/example_scenario.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\PythonProjects\aiphoria\tests\reference_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE8631F8-DCCB-44A2-B43F-6A78958E5BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02CCFECC-5257-49F4-A9AD-27E890745104}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1000A452-A98F-45C1-B843-91F7F67E097C}"/>
   </bookViews>
   <sheets>
     <sheet name="Settings" sheetId="11" r:id="rId1"/>
@@ -49,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="232">
   <si>
     <t>Years</t>
   </si>
@@ -783,6 +783,12 @@
   </si>
   <si>
     <t>prioritize_transformation_stages</t>
+  </si>
+  <si>
+    <t>version</t>
+  </si>
+  <si>
+    <t>Scenario file version</t>
   </si>
 </sst>
 </file>
@@ -926,7 +932,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -960,6 +966,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1422,7 +1429,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89FFA668-DA1A-459B-BD42-D0D7F7709F0D}">
-  <dimension ref="A2:E41"/>
+  <dimension ref="A2:E42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.7109375" bestFit="1" customWidth="1"/>
@@ -1466,173 +1473,170 @@
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" s="20" t="s">
-        <v>1</v>
+        <v>230</v>
+      </c>
+      <c r="C7" s="19">
+        <v>2</v>
       </c>
       <c r="D7" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="E7" t="s">
-        <v>228</v>
+      <c r="E7" s="23" t="s">
+        <v>231</v>
       </c>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>146</v>
-      </c>
-      <c r="C8" t="s">
-        <v>172</v>
-      </c>
-      <c r="D8" t="s">
-        <v>121</v>
+        <v>60</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>88</v>
       </c>
       <c r="E8" t="s">
-        <v>148</v>
+        <v>228</v>
       </c>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="19">
-        <v>2</v>
-      </c>
-      <c r="D9" s="19" t="s">
-        <v>86</v>
+        <v>146</v>
+      </c>
+      <c r="C9" t="s">
+        <v>172</v>
+      </c>
+      <c r="D9" t="s">
+        <v>121</v>
       </c>
       <c r="E9" t="s">
-        <v>64</v>
+        <v>148</v>
       </c>
     </row>
     <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>62</v>
-      </c>
-      <c r="C10" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" s="19">
         <v>2</v>
       </c>
-      <c r="D10" s="20" t="s">
-        <v>87</v>
+      <c r="D10" s="19" t="s">
+        <v>86</v>
       </c>
       <c r="E10" t="s">
-        <v>227</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>147</v>
-      </c>
-      <c r="C11" t="s">
-        <v>172</v>
-      </c>
-      <c r="D11" t="s">
-        <v>121</v>
+        <v>62</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>87</v>
       </c>
       <c r="E11" t="s">
-        <v>149</v>
+        <v>227</v>
       </c>
     </row>
     <row r="12" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>63</v>
-      </c>
-      <c r="C12" s="19">
-        <v>2</v>
-      </c>
-      <c r="D12" s="19" t="s">
-        <v>86</v>
+        <v>147</v>
+      </c>
+      <c r="C12" t="s">
+        <v>172</v>
+      </c>
+      <c r="D12" t="s">
+        <v>121</v>
       </c>
       <c r="E12" t="s">
-        <v>64</v>
+        <v>149</v>
       </c>
     </row>
     <row r="13" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C13" s="19">
-        <v>2021</v>
+        <v>2</v>
       </c>
       <c r="D13" s="19" t="s">
         <v>86</v>
       </c>
       <c r="E13" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C14" s="19">
-        <v>2030</v>
+        <v>2021</v>
       </c>
       <c r="D14" s="19" t="s">
         <v>86</v>
       </c>
       <c r="E14" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
     </row>
     <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>68</v>
-      </c>
-      <c r="C15" s="21" t="b">
-        <v>0</v>
-      </c>
-      <c r="D15" t="s">
-        <v>85</v>
+        <v>67</v>
+      </c>
+      <c r="C15" s="19">
+        <v>2030</v>
+      </c>
+      <c r="D15" s="19" t="s">
+        <v>86</v>
       </c>
       <c r="E15" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C16" s="21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D16" t="s">
         <v>85</v>
       </c>
       <c r="E16" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
+        <v>71</v>
+      </c>
+      <c r="C17" s="21" t="b">
+        <v>1</v>
+      </c>
+      <c r="D17" t="s">
+        <v>85</v>
+      </c>
+      <c r="E17" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B18" t="s">
         <v>79</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C18" s="11">
         <v>0.1</v>
       </c>
-      <c r="D17" s="19" t="s">
+      <c r="D18" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E18" t="s">
         <v>80</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>189</v>
-      </c>
-      <c r="B18" t="s">
-        <v>163</v>
-      </c>
-      <c r="C18" t="s">
-        <v>171</v>
-      </c>
-      <c r="D18" t="s">
-        <v>87</v>
-      </c>
-      <c r="E18" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -1640,16 +1644,16 @@
         <v>189</v>
       </c>
       <c r="B19" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C19" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="D19" t="s">
         <v>87</v>
       </c>
       <c r="E19" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -1657,16 +1661,16 @@
         <v>189</v>
       </c>
       <c r="B20" t="s">
-        <v>73</v>
-      </c>
-      <c r="C20" s="17">
-        <v>-3.6666666666666701</v>
-      </c>
-      <c r="D20" s="17" t="s">
-        <v>89</v>
+        <v>164</v>
+      </c>
+      <c r="C20" t="s">
+        <v>167</v>
+      </c>
+      <c r="D20" t="s">
+        <v>87</v>
       </c>
       <c r="E20" t="s">
-        <v>74</v>
+        <v>165</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -1674,16 +1678,16 @@
         <v>189</v>
       </c>
       <c r="B21" t="s">
-        <v>83</v>
-      </c>
-      <c r="C21" s="21" t="b">
-        <v>1</v>
-      </c>
-      <c r="D21" t="s">
-        <v>85</v>
+        <v>73</v>
+      </c>
+      <c r="C21" s="17">
+        <v>-3.6666666666666701</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>89</v>
       </c>
       <c r="E21" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1691,7 +1695,7 @@
         <v>189</v>
       </c>
       <c r="B22" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C22" s="21" t="b">
         <v>1</v>
@@ -1708,16 +1712,16 @@
         <v>189</v>
       </c>
       <c r="B23" t="s">
-        <v>90</v>
-      </c>
-      <c r="C23" t="s">
-        <v>93</v>
+        <v>82</v>
+      </c>
+      <c r="C23" s="21" t="b">
+        <v>1</v>
       </c>
       <c r="D23" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E23" t="s">
-        <v>111</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -1725,16 +1729,16 @@
         <v>189</v>
       </c>
       <c r="B24" t="s">
-        <v>175</v>
-      </c>
-      <c r="C24" s="21" t="b">
-        <v>1</v>
+        <v>90</v>
+      </c>
+      <c r="C24" t="s">
+        <v>93</v>
       </c>
       <c r="D24" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="E24" t="s">
-        <v>176</v>
+        <v>111</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -1742,16 +1746,16 @@
         <v>189</v>
       </c>
       <c r="B25" t="s">
-        <v>184</v>
-      </c>
-      <c r="C25" t="s">
-        <v>186</v>
+        <v>175</v>
+      </c>
+      <c r="C25" s="21" t="b">
+        <v>1</v>
       </c>
       <c r="D25" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E25" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -1759,16 +1763,16 @@
         <v>189</v>
       </c>
       <c r="B26" t="s">
-        <v>96</v>
+        <v>184</v>
       </c>
       <c r="C26" t="s">
-        <v>97</v>
+        <v>186</v>
       </c>
       <c r="D26" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E26" t="s">
-        <v>226</v>
+        <v>188</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -1776,13 +1780,16 @@
         <v>189</v>
       </c>
       <c r="B27" t="s">
-        <v>153</v>
+        <v>96</v>
+      </c>
+      <c r="C27" t="s">
+        <v>97</v>
       </c>
       <c r="D27" t="s">
-        <v>121</v>
+        <v>87</v>
       </c>
       <c r="E27" t="s">
-        <v>155</v>
+        <v>226</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -1790,16 +1797,13 @@
         <v>189</v>
       </c>
       <c r="B28" t="s">
-        <v>98</v>
-      </c>
-      <c r="C28" s="21" t="b">
-        <v>1</v>
+        <v>153</v>
       </c>
       <c r="D28" t="s">
-        <v>85</v>
+        <v>121</v>
       </c>
       <c r="E28" t="s">
-        <v>99</v>
+        <v>155</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1807,7 +1811,7 @@
         <v>189</v>
       </c>
       <c r="B29" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C29" s="21" t="b">
         <v>1</v>
@@ -1816,7 +1820,7 @@
         <v>85</v>
       </c>
       <c r="E29" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -1824,16 +1828,16 @@
         <v>189</v>
       </c>
       <c r="B30" t="s">
-        <v>119</v>
-      </c>
-      <c r="C30" t="s">
-        <v>122</v>
+        <v>100</v>
+      </c>
+      <c r="C30" s="21" t="b">
+        <v>1</v>
       </c>
       <c r="D30" t="s">
-        <v>121</v>
+        <v>85</v>
       </c>
       <c r="E30" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
@@ -1841,16 +1845,16 @@
         <v>189</v>
       </c>
       <c r="B31" t="s">
-        <v>139</v>
-      </c>
-      <c r="C31" s="19" t="s">
-        <v>140</v>
-      </c>
-      <c r="D31" s="19" t="s">
-        <v>87</v>
+        <v>119</v>
+      </c>
+      <c r="C31" t="s">
+        <v>122</v>
+      </c>
+      <c r="D31" t="s">
+        <v>121</v>
       </c>
       <c r="E31" t="s">
-        <v>225</v>
+        <v>120</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -1858,41 +1862,44 @@
         <v>189</v>
       </c>
       <c r="B32" t="s">
-        <v>154</v>
-      </c>
-      <c r="D32" t="s">
-        <v>121</v>
+        <v>139</v>
+      </c>
+      <c r="C32" s="19" t="s">
+        <v>140</v>
+      </c>
+      <c r="D32" s="19" t="s">
+        <v>87</v>
       </c>
       <c r="E32" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>189</v>
       </c>
       <c r="B33" t="s">
-        <v>178</v>
+        <v>154</v>
       </c>
       <c r="D33" t="s">
         <v>121</v>
       </c>
       <c r="E33" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>189</v>
       </c>
       <c r="B34" t="s">
-        <v>229</v>
+        <v>178</v>
       </c>
       <c r="D34" t="s">
         <v>121</v>
       </c>
       <c r="E34" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1900,16 +1907,13 @@
         <v>189</v>
       </c>
       <c r="B35" t="s">
-        <v>190</v>
-      </c>
-      <c r="C35" t="s">
-        <v>191</v>
+        <v>229</v>
       </c>
       <c r="D35" t="s">
-        <v>87</v>
+        <v>121</v>
       </c>
       <c r="E35" t="s">
-        <v>224</v>
+        <v>180</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1917,16 +1921,16 @@
         <v>189</v>
       </c>
       <c r="B36" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="C36" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="D36" t="s">
         <v>87</v>
       </c>
       <c r="E36" t="s">
-        <v>202</v>
+        <v>224</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -1934,16 +1938,16 @@
         <v>189</v>
       </c>
       <c r="B37" t="s">
-        <v>203</v>
-      </c>
-      <c r="C37" s="21" t="b">
-        <v>1</v>
+        <v>200</v>
+      </c>
+      <c r="C37" t="s">
+        <v>201</v>
       </c>
       <c r="D37" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="E37" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
@@ -1951,7 +1955,7 @@
         <v>189</v>
       </c>
       <c r="B38" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="C38" s="21" t="b">
         <v>1</v>
@@ -1960,7 +1964,7 @@
         <v>85</v>
       </c>
       <c r="E38" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -1968,16 +1972,16 @@
         <v>189</v>
       </c>
       <c r="B39" t="s">
-        <v>217</v>
-      </c>
-      <c r="C39" t="s">
-        <v>218</v>
+        <v>215</v>
+      </c>
+      <c r="C39" s="21" t="b">
+        <v>1</v>
       </c>
       <c r="D39" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E39" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1985,16 +1989,16 @@
         <v>189</v>
       </c>
       <c r="B40" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C40" t="s">
-        <v>172</v>
+        <v>218</v>
       </c>
       <c r="D40" t="s">
-        <v>121</v>
+        <v>87</v>
       </c>
       <c r="E40" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -2002,21 +2006,38 @@
         <v>189</v>
       </c>
       <c r="B41" t="s">
+        <v>219</v>
+      </c>
+      <c r="C41" t="s">
+        <v>172</v>
+      </c>
+      <c r="D41" t="s">
+        <v>121</v>
+      </c>
+      <c r="E41" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>189</v>
+      </c>
+      <c r="B42" t="s">
         <v>221</v>
       </c>
-      <c r="C41">
+      <c r="C42">
         <v>2</v>
       </c>
-      <c r="D41" t="s">
+      <c r="D42" t="s">
         <v>86</v>
       </c>
-      <c r="E41" t="s">
+      <c r="E42" t="s">
         <v>222</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="B6:E6" xr:uid="{89FFA668-DA1A-459B-BD42-D0D7F7709F0D}"/>
-  <conditionalFormatting sqref="C15:C16">
+  <conditionalFormatting sqref="C16:C17">
     <cfRule type="cellIs" dxfId="11" priority="11" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -2024,7 +2045,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C21:C22">
+  <conditionalFormatting sqref="C22:C23">
     <cfRule type="cellIs" dxfId="9" priority="9" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -2032,7 +2053,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C24">
+  <conditionalFormatting sqref="C25">
     <cfRule type="cellIs" dxfId="7" priority="5" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -2040,7 +2061,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C28:C29">
+  <conditionalFormatting sqref="C29:C30">
     <cfRule type="cellIs" dxfId="5" priority="7" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -2048,7 +2069,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C37:C38">
+  <conditionalFormatting sqref="C38:C39">
     <cfRule type="cellIs" dxfId="3" priority="3" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
@@ -2057,7 +2078,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C15:C16 C21:C22 C28:C29 C24 C37:C38" xr:uid="{79A7E31C-3284-4405-9B5F-03E099B07563}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C16:C17 C22:C23 C29:C30 C25 C38:C39" xr:uid="{79A7E31C-3284-4405-9B5F-03E099B07563}">
       <formula1>Boolean</formula1>
     </dataValidation>
   </dataValidations>
@@ -2070,13 +2091,13 @@
           <x14:formula1>
             <xm:f>'Data validation parameters'!$D$6:$D$9</xm:f>
           </x14:formula1>
-          <xm:sqref>C23</xm:sqref>
+          <xm:sqref>C24</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7A04E2A2-4928-4E28-9F6D-7D556381B8E8}">
           <x14:formula1>
             <xm:f>'Data validation parameters'!$G$6:$G$7</xm:f>
           </x14:formula1>
-          <xm:sqref>C25</xm:sqref>
+          <xm:sqref>C26</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -5182,18 +5203,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="145cc194-9bea-4db6-b116-a042a4529fcd" xsi:nil="true"/>
-    <Comment xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Asiakirja" ma:contentTypeID="0x010100806C55B750152A459818B636E97A41C3" ma:contentTypeVersion="19" ma:contentTypeDescription="Luo uusi asiakirja." ma:contentTypeScope="" ma:versionID="74fd9cb75cef04cf26a1ff9ddef01b4b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7536dd80-7d39-48e8-9ae3-b4166f580a2d" xmlns:ns3="145cc194-9bea-4db6-b116-a042a4529fcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="afbcbfdd38894bc2ff0644b00c8ec680" ns2:_="" ns3:_="">
     <xsd:import namespace="7536dd80-7d39-48e8-9ae3-b4166f580a2d"/>
@@ -5456,6 +5465,18 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="145cc194-9bea-4db6-b116-a042a4529fcd" xsi:nil="true"/>
+    <Comment xmlns="7536dd80-7d39-48e8-9ae3-b4166f580a2d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AB3C6F0-DB35-46F0-8FEB-B5E57B48A727}">
   <ds:schemaRefs>
@@ -5465,23 +5486,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{557FAA9C-B184-448F-B58D-00E4D46BDD72}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="7536dd80-7d39-48e8-9ae3-b4166f580a2d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="145cc194-9bea-4db6-b116-a042a4529fcd"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D60021C7-CA75-4673-96EA-55284BF81134}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5498,4 +5502,21 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{557FAA9C-B184-448F-B58D-00E4D46BDD72}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="7536dd80-7d39-48e8-9ae3-b4166f580a2d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="145cc194-9bea-4db6-b116-a042a4529fcd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>